<commit_message>
ECS-93 added hyperlinks in evaluation-logs and experiments xlsx reports
</commit_message>
<xml_diff>
--- a/eca-server/src/main/resources/report-templates/evaluation-logs-report-template.xlsx
+++ b/eca-server/src/main/resources/report-templates/evaluation-logs-report-template.xlsx
@@ -306,9 +306,6 @@
     <t>Дата удаления модели</t>
   </si>
   <si>
-    <t>${evaluationLog.requestId}</t>
-  </si>
-  <si>
     <t>${evaluationLog.classifierName}</t>
   </si>
   <si>
@@ -377,6 +374,9 @@
   </si>
   <si>
     <t>${filter.description}</t>
+  </si>
+  <si>
+    <t>${util.hyperlink(evaluationLog.externalDetailsUrl, evaluationLog.requestId)}</t>
   </si>
 </sst>
 </file>
@@ -533,9 +533,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -543,6 +540,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -821,7 +821,7 @@
       <c r="M2" s="2"/>
     </row>
     <row r="3" spans="1:18" ht="14.85" customHeight="1">
-      <c r="A3" s="10" t="s">
+      <c r="A3" s="9" t="s">
         <v>1</v>
       </c>
       <c r="B3" s="12" t="s">
@@ -841,7 +841,7 @@
     </row>
     <row r="4" spans="1:18" ht="14.85" customHeight="1">
       <c r="A4" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B4" s="16" t="s">
         <v>4</v>
@@ -958,49 +958,49 @@
       <c r="R8" s="6"/>
     </row>
     <row r="9" spans="1:18" ht="15" customHeight="1">
-      <c r="A9" s="7" t="s">
+      <c r="A9" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="B9" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="C9" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="C9" s="8" t="s">
+      <c r="D9" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="D9" s="8" t="s">
+      <c r="E9" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="E9" s="8" t="s">
+      <c r="F9" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="F9" s="8" t="s">
+      <c r="G9" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G9" s="8" t="s">
+      <c r="H9" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="H9" s="8" t="s">
+      <c r="I9" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="I9" s="8" t="s">
+      <c r="J9" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="J9" s="8" t="s">
+      <c r="K9" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="K9" s="9" t="s">
+      <c r="L9" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="L9" s="8" t="s">
+      <c r="M9" s="7" t="s">
         <v>31</v>
-      </c>
-      <c r="M9" s="8" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="10" spans="1:18">
       <c r="A10" s="13" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B10" s="14"/>
       <c r="C10" s="14"/>

</xml_diff>

<commit_message>
ECS-98 added extended instances info in evaluation-logs-report-template.xlsx, experiments-report-template.xlsx
</commit_message>
<xml_diff>
--- a/eca-server/src/main/resources/report-templates/evaluation-logs-report-template.xlsx
+++ b/eca-server/src/main/resources/report-templates/evaluation-logs-report-template.xlsx
@@ -319,9 +319,6 @@
     </r>
   </si>
   <si>
-    <t>${evaluationLog.relationName}</t>
-  </si>
-  <si>
     <t>${evaluationLog.evaluationMethod}</t>
   </si>
   <si>
@@ -400,6 +397,13 @@
       <t xml:space="preserve">
 ${evaluationLog.classifierOptions}</t>
     </r>
+  </si>
+  <si>
+    <t>${evaluationLog.relationName}
+Число объектов: ${evaluationLog.numInstances}
+Число атрибутов: ${evaluationLog.numAttributes}
+Число классов: ${evaluationLog.numClasses}
+Атрибут класса: ${evaluationLog.className}</t>
   </si>
 </sst>
 </file>
@@ -581,6 +585,9 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -589,9 +596,6 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -830,21 +834,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="15.6">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="11"/>
-      <c r="H1" s="11"/>
-      <c r="I1" s="11"/>
-      <c r="J1" s="11"/>
-      <c r="K1" s="11"/>
-      <c r="L1" s="11"/>
-      <c r="M1" s="11"/>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12"/>
+      <c r="H1" s="12"/>
+      <c r="I1" s="12"/>
+      <c r="J1" s="12"/>
+      <c r="K1" s="12"/>
+      <c r="L1" s="12"/>
+      <c r="M1" s="12"/>
     </row>
     <row r="2" spans="1:18" ht="15.6">
       <c r="A2" s="1"/>
@@ -865,77 +869,77 @@
       <c r="A3" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="12" t="s">
+      <c r="B3" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="12"/>
-      <c r="D3" s="12"/>
-      <c r="E3" s="12"/>
-      <c r="F3" s="12"/>
-      <c r="G3" s="12"/>
-      <c r="H3" s="12"/>
-      <c r="I3" s="12"/>
-      <c r="J3" s="12"/>
-      <c r="K3" s="12"/>
-      <c r="L3" s="12"/>
-      <c r="M3" s="12"/>
+      <c r="C3" s="13"/>
+      <c r="D3" s="13"/>
+      <c r="E3" s="13"/>
+      <c r="F3" s="13"/>
+      <c r="G3" s="13"/>
+      <c r="H3" s="13"/>
+      <c r="I3" s="13"/>
+      <c r="J3" s="13"/>
+      <c r="K3" s="13"/>
+      <c r="L3" s="13"/>
+      <c r="M3" s="13"/>
     </row>
     <row r="4" spans="1:18" ht="14.85" customHeight="1">
       <c r="A4" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="B4" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="B4" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="16"/>
-      <c r="D4" s="16"/>
-      <c r="E4" s="16"/>
-      <c r="F4" s="16"/>
-      <c r="G4" s="16"/>
-      <c r="H4" s="16"/>
-      <c r="I4" s="16"/>
-      <c r="J4" s="16"/>
-      <c r="K4" s="16"/>
-      <c r="L4" s="16"/>
-      <c r="M4" s="16"/>
+      <c r="C4" s="17"/>
+      <c r="D4" s="17"/>
+      <c r="E4" s="17"/>
+      <c r="F4" s="17"/>
+      <c r="G4" s="17"/>
+      <c r="H4" s="17"/>
+      <c r="I4" s="17"/>
+      <c r="J4" s="17"/>
+      <c r="K4" s="17"/>
+      <c r="L4" s="17"/>
+      <c r="M4" s="17"/>
     </row>
     <row r="5" spans="1:18" ht="14.85" customHeight="1">
       <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="16" t="s">
+      <c r="B5" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="16"/>
-      <c r="D5" s="16"/>
-      <c r="E5" s="16"/>
-      <c r="F5" s="16"/>
-      <c r="G5" s="16"/>
-      <c r="H5" s="16"/>
-      <c r="I5" s="16"/>
-      <c r="J5" s="16"/>
-      <c r="K5" s="16"/>
-      <c r="L5" s="16"/>
-      <c r="M5" s="16"/>
+      <c r="C5" s="17"/>
+      <c r="D5" s="17"/>
+      <c r="E5" s="17"/>
+      <c r="F5" s="17"/>
+      <c r="G5" s="17"/>
+      <c r="H5" s="17"/>
+      <c r="I5" s="17"/>
+      <c r="J5" s="17"/>
+      <c r="K5" s="17"/>
+      <c r="L5" s="17"/>
+      <c r="M5" s="17"/>
     </row>
     <row r="6" spans="1:18" ht="14.85" customHeight="1">
       <c r="A6" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="16" t="s">
+      <c r="B6" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="16"/>
-      <c r="D6" s="16"/>
-      <c r="E6" s="16"/>
-      <c r="F6" s="16"/>
-      <c r="G6" s="16"/>
-      <c r="H6" s="16"/>
-      <c r="I6" s="16"/>
-      <c r="J6" s="16"/>
-      <c r="K6" s="16"/>
-      <c r="L6" s="16"/>
-      <c r="M6" s="16"/>
+      <c r="C6" s="17"/>
+      <c r="D6" s="17"/>
+      <c r="E6" s="17"/>
+      <c r="F6" s="17"/>
+      <c r="G6" s="17"/>
+      <c r="H6" s="17"/>
+      <c r="I6" s="17"/>
+      <c r="J6" s="17"/>
+      <c r="K6" s="17"/>
+      <c r="L6" s="17"/>
+      <c r="M6" s="17"/>
     </row>
     <row r="7" spans="1:18">
       <c r="A7" s="2"/>
@@ -1000,10 +1004,10 @@
     </row>
     <row r="9" spans="1:18" ht="15" customHeight="1">
       <c r="A9" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="B9" s="11" t="s">
         <v>33</v>
-      </c>
-      <c r="B9" s="17" t="s">
-        <v>34</v>
       </c>
       <c r="C9" s="7" t="s">
         <v>20</v>
@@ -1011,50 +1015,50 @@
       <c r="D9" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="E9" s="7" t="s">
+      <c r="E9" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="F9" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="F9" s="7" t="s">
+      <c r="G9" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="G9" s="7" t="s">
+      <c r="H9" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="H9" s="7" t="s">
+      <c r="I9" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="I9" s="7" t="s">
+      <c r="J9" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="J9" s="7" t="s">
+      <c r="K9" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="K9" s="8" t="s">
+      <c r="L9" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="L9" s="7" t="s">
+      <c r="M9" s="7" t="s">
         <v>29</v>
-      </c>
-      <c r="M9" s="7" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="10" spans="1:18">
-      <c r="A10" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="B10" s="14"/>
-      <c r="C10" s="14"/>
-      <c r="D10" s="14"/>
-      <c r="E10" s="14"/>
-      <c r="F10" s="14"/>
-      <c r="G10" s="14"/>
-      <c r="H10" s="14"/>
-      <c r="I10" s="14"/>
-      <c r="J10" s="14"/>
-      <c r="K10" s="14"/>
-      <c r="L10" s="14"/>
-      <c r="M10" s="15"/>
+      <c r="A10" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="B10" s="15"/>
+      <c r="C10" s="15"/>
+      <c r="D10" s="15"/>
+      <c r="E10" s="15"/>
+      <c r="F10" s="15"/>
+      <c r="G10" s="15"/>
+      <c r="H10" s="15"/>
+      <c r="I10" s="15"/>
+      <c r="J10" s="15"/>
+      <c r="K10" s="15"/>
+      <c r="L10" s="15"/>
+      <c r="M10" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="6">

</xml_diff>